<commit_message>
add private cetak sk sp
</commit_message>
<xml_diff>
--- a/public/template/template_riwayat_kerja.xlsx
+++ b/public/template/template_riwayat_kerja.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="9">
   <si>
     <t>No</t>
   </si>
@@ -43,106 +43,13 @@
   <si>
     <t>Tahun</t>
   </si>
-  <si>
-    <t>PG250518171715</t>
-  </si>
-  <si>
-    <t>PG250521769296</t>
-  </si>
-  <si>
-    <t>PG250521769297</t>
-  </si>
-  <si>
-    <t>PG250521179441</t>
-  </si>
-  <si>
-    <t>PG250604463155</t>
-  </si>
-  <si>
-    <t>PG250604463156</t>
-  </si>
-  <si>
-    <t>PG250604463157</t>
-  </si>
-  <si>
-    <t>PG250604463158</t>
-  </si>
-  <si>
-    <t>PG250604463159</t>
-  </si>
-  <si>
-    <t>PG250604463160</t>
-  </si>
-  <si>
-    <t>PG250604463161</t>
-  </si>
-  <si>
-    <t>PG250604463162</t>
-  </si>
-  <si>
-    <t>FAJAR AJI KUSUMA</t>
-  </si>
-  <si>
-    <t>MEILIYA ISMIYATI</t>
-  </si>
-  <si>
-    <t>MUROHATI</t>
-  </si>
-  <si>
-    <t>BAGUS JIWAN NIZAL SAPUTRA</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>H</t>
-  </si>
-  <si>
-    <t>Tenaga Administrasi</t>
-  </si>
-  <si>
-    <t>Akuntan</t>
-  </si>
-  <si>
-    <t>Desainer Grafis</t>
-  </si>
-  <si>
-    <t>Sekretariat</t>
-  </si>
-  <si>
-    <t>KPS</t>
-  </si>
-  <si>
-    <t>PPKL</t>
-  </si>
-  <si>
-    <t>Taling</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -154,15 +61,6 @@
     </font>
     <font>
       <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b val="0"/>
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
@@ -206,20 +104,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="true">
       <protection locked="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-      <protection locked="true"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-      <protection locked="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
       <protection locked="true"/>
     </xf>
@@ -524,17 +414,6 @@
   </sheetPr>
   <dimension ref="A1:I900"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col min="1" max="1" width="5" customWidth="true" style="0"/>
-    <col min="2" max="2" width="15" customWidth="true" style="0"/>
-    <col min="3" max="3" width="25" customWidth="true" style="0"/>
-    <col min="4" max="4" width="20" customWidth="true" style="0"/>
-    <col min="5" max="5" width="20" customWidth="true" style="0"/>
-    <col min="6" max="6" width="15" customWidth="true" style="0"/>
-    <col min="7" max="7" width="15" customWidth="true" style="0"/>
-    <col min="8" max="8" width="15" customWidth="true" style="0"/>
-    <col min="9" max="9" width="10" customWidth="true" style="0"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="2" t="s">
@@ -565,293 +444,137 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" customHeight="1" ht="20">
-      <c r="A2" s="3">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="4" t="e">
-        <f>YEAR(F2)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" customHeight="1" ht="20">
-      <c r="A3" s="3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="4" t="e">
-        <f>YEAR(F3)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" customHeight="1" ht="20">
-      <c r="A4" s="3">
-        <v>3</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="4" t="e">
-        <f>YEAR(F4)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" customHeight="1" ht="20">
-      <c r="A5" s="3">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="4" t="e">
-        <f>YEAR(F5)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" customHeight="1" ht="20">
-      <c r="A6" s="3">
-        <v>5</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="4" t="e">
-        <f>YEAR(F6)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" customHeight="1" ht="20">
-      <c r="A7" s="3">
-        <v>6</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="4" t="e">
-        <f>YEAR(F7)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" customHeight="1" ht="20">
-      <c r="A8" s="3">
-        <v>7</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="4" t="e">
-        <f>YEAR(F8)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" customHeight="1" ht="20">
-      <c r="A9" s="3">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="4" t="e">
-        <f>YEAR(F9)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" customHeight="1" ht="20">
-      <c r="A10" s="3">
-        <v>9</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="4" t="e">
-        <f>YEAR(F10)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" customHeight="1" ht="20">
-      <c r="A11" s="3">
-        <v>10</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="4" t="e">
-        <f>YEAR(F11)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" customHeight="1" ht="20">
-      <c r="A12" s="3">
-        <v>11</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="4" t="e">
-        <f>YEAR(F12)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" customHeight="1" ht="20">
-      <c r="A13" s="3">
-        <v>12</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="4" t="e">
-        <f>YEAR(F13)</f>
-        <v>#VALUE!</v>
-      </c>
+    <row r="2" spans="1:9">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="1"/>
@@ -10612,140 +10335,6 @@
     </row>
   </sheetData>
   <sheetProtection password="9D39" sheet="1"/>
-  <dataValidations count="60">
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D2">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E2">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F2"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G2"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H2">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D3">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E3">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F3"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G3"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H3">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D4">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E4">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F4"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G4"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H4">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D5">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E5">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F5"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G5"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H5">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D6">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E6">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F6"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G6"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H6">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D7">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E7">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F7"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G7"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H7">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D8">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E8">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F8"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G8"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H8">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D9">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E9">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F9"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G9"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H9">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D10">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E10">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F10"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G10"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H10">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D11">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E11">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F11"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G11"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H11">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D12">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E12">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F12"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G12"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H12">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D13">
-      <formula1>"Tenaga Administrasi,Petugas Angkutan Sampah,Marketing,Programmer,Desainer Grafis,Customer Service,Akuntan,HRD,Content Writer,Teknisi IT,Supervisor,Administrator,Tukang Sapu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E13">
-      <formula1>"Sekretariat,Taling,KPS,PPKL"</formula1>
-    </dataValidation>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F13"/>
-    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G13"/>
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H13">
-      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
-    </dataValidation>
-  </dataValidations>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>

</xml_diff>

<commit_message>
versi lama 12 Juli 2026
</commit_message>
<xml_diff>
--- a/public/template/template_riwayat_kerja.xlsx
+++ b/public/template/template_riwayat_kerja.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="144">
   <si>
     <t>No</t>
   </si>
@@ -42,6 +42,411 @@
   </si>
   <si>
     <t>Tahun</t>
+  </si>
+  <si>
+    <t>PG260109252897</t>
+  </si>
+  <si>
+    <t>PG260109252898</t>
+  </si>
+  <si>
+    <t>PG260109252901</t>
+  </si>
+  <si>
+    <t>PG260109252902</t>
+  </si>
+  <si>
+    <t>PG260109252904</t>
+  </si>
+  <si>
+    <t>PG260109252905</t>
+  </si>
+  <si>
+    <t>PG260109252906</t>
+  </si>
+  <si>
+    <t>PG260109252907</t>
+  </si>
+  <si>
+    <t>PG260109252908</t>
+  </si>
+  <si>
+    <t>PG260109252909</t>
+  </si>
+  <si>
+    <t>PG260109252910</t>
+  </si>
+  <si>
+    <t>PG260109252911</t>
+  </si>
+  <si>
+    <t>PG260109252912</t>
+  </si>
+  <si>
+    <t>PG260109252913</t>
+  </si>
+  <si>
+    <t>PG260109252914</t>
+  </si>
+  <si>
+    <t>PG260109252915</t>
+  </si>
+  <si>
+    <t>PG260109252916</t>
+  </si>
+  <si>
+    <t>PG260109252918</t>
+  </si>
+  <si>
+    <t>PG260109252919</t>
+  </si>
+  <si>
+    <t>PG260109252920</t>
+  </si>
+  <si>
+    <t>PG260109252921</t>
+  </si>
+  <si>
+    <t>PG260109252922</t>
+  </si>
+  <si>
+    <t>PG260109252923</t>
+  </si>
+  <si>
+    <t>PG260109252924</t>
+  </si>
+  <si>
+    <t>PG260109252925</t>
+  </si>
+  <si>
+    <t>PG260109252926</t>
+  </si>
+  <si>
+    <t>PG260109252927</t>
+  </si>
+  <si>
+    <t>PG260109252928</t>
+  </si>
+  <si>
+    <t>PG260109252929</t>
+  </si>
+  <si>
+    <t>PG260109252930</t>
+  </si>
+  <si>
+    <t>PG260109252931</t>
+  </si>
+  <si>
+    <t>PG260109252932</t>
+  </si>
+  <si>
+    <t>PG260109252933</t>
+  </si>
+  <si>
+    <t>PG260109252934</t>
+  </si>
+  <si>
+    <t>PG260109252935</t>
+  </si>
+  <si>
+    <t>PG260109252936</t>
+  </si>
+  <si>
+    <t>PG260109252937</t>
+  </si>
+  <si>
+    <t>PG260109252938</t>
+  </si>
+  <si>
+    <t>PG260109252939</t>
+  </si>
+  <si>
+    <t>PG260109252941</t>
+  </si>
+  <si>
+    <t>PG260109252944</t>
+  </si>
+  <si>
+    <t>PG260109252946</t>
+  </si>
+  <si>
+    <t>PG260109252947</t>
+  </si>
+  <si>
+    <t>PG260109252948</t>
+  </si>
+  <si>
+    <t>PG260109252949</t>
+  </si>
+  <si>
+    <t>PG260109252950</t>
+  </si>
+  <si>
+    <t>PG260109252951</t>
+  </si>
+  <si>
+    <t>PG260109252952</t>
+  </si>
+  <si>
+    <t>PG260109252953</t>
+  </si>
+  <si>
+    <t>PG260109252954</t>
+  </si>
+  <si>
+    <t>PG260109252955</t>
+  </si>
+  <si>
+    <t>PG260109252956</t>
+  </si>
+  <si>
+    <t>PG260109252957</t>
+  </si>
+  <si>
+    <t>PG260109252958</t>
+  </si>
+  <si>
+    <t>PG260109252959</t>
+  </si>
+  <si>
+    <t>PG260109252960</t>
+  </si>
+  <si>
+    <t>PG260109252961</t>
+  </si>
+  <si>
+    <t>PG260109252962</t>
+  </si>
+  <si>
+    <t>PG260129995530</t>
+  </si>
+  <si>
+    <t>Fajar Aji Kusuma</t>
+  </si>
+  <si>
+    <t>Triono</t>
+  </si>
+  <si>
+    <t>Muhammad Tomy Abdul Haris</t>
+  </si>
+  <si>
+    <t>Bambang Setiaji</t>
+  </si>
+  <si>
+    <t>Friessanti Adi Valindyasari</t>
+  </si>
+  <si>
+    <t>Chafidh Rochmatullah</t>
+  </si>
+  <si>
+    <t>Kalimin</t>
+  </si>
+  <si>
+    <t>Mursalin</t>
+  </si>
+  <si>
+    <t>Iwan Santosa</t>
+  </si>
+  <si>
+    <t>Ali Akbar</t>
+  </si>
+  <si>
+    <t>Nurmalita</t>
+  </si>
+  <si>
+    <t>Sri Wijayanti</t>
+  </si>
+  <si>
+    <t>Slamet Muzafak</t>
+  </si>
+  <si>
+    <t>Purwati</t>
+  </si>
+  <si>
+    <t>Asrofudin</t>
+  </si>
+  <si>
+    <t>Muchammad Fariz</t>
+  </si>
+  <si>
+    <t>Zaenal</t>
+  </si>
+  <si>
+    <t>Muhammad Muttaqin</t>
+  </si>
+  <si>
+    <t>Sabila Oktaviani Putri</t>
+  </si>
+  <si>
+    <t>Widiyanto</t>
+  </si>
+  <si>
+    <t>Radna Pambudhi</t>
+  </si>
+  <si>
+    <t>Fatchurohman</t>
+  </si>
+  <si>
+    <t>Anita Uslifa</t>
+  </si>
+  <si>
+    <t>Masro'ah</t>
+  </si>
+  <si>
+    <t>Slamet Mulyono</t>
+  </si>
+  <si>
+    <t>Arif Budiono</t>
+  </si>
+  <si>
+    <t>Sutaji</t>
+  </si>
+  <si>
+    <t>Ady Laksono</t>
+  </si>
+  <si>
+    <t>Indah Elliana</t>
+  </si>
+  <si>
+    <t>Taufik Rahman</t>
+  </si>
+  <si>
+    <t>Agung Wibowo</t>
+  </si>
+  <si>
+    <t>Irfan Ali</t>
+  </si>
+  <si>
+    <t>Nurochim</t>
+  </si>
+  <si>
+    <t>Khaerul Umam</t>
+  </si>
+  <si>
+    <t>Zamproni</t>
+  </si>
+  <si>
+    <t>Achmad Zakaria</t>
+  </si>
+  <si>
+    <t>Suprianto</t>
+  </si>
+  <si>
+    <t>Galih Prasetya</t>
+  </si>
+  <si>
+    <t>Reza Yahya</t>
+  </si>
+  <si>
+    <t>Nidhom Adinata</t>
+  </si>
+  <si>
+    <t>Jamal Adi Prasetiyo</t>
+  </si>
+  <si>
+    <t>Rizqi Tri Atmaja</t>
+  </si>
+  <si>
+    <t>Dhimas Abimanyu</t>
+  </si>
+  <si>
+    <t>Esti Herti</t>
+  </si>
+  <si>
+    <t>Edy Santoso</t>
+  </si>
+  <si>
+    <t>Saiful Bahri</t>
+  </si>
+  <si>
+    <t>Choirul Umam</t>
+  </si>
+  <si>
+    <t>Aulia Triska Prasojo</t>
+  </si>
+  <si>
+    <t>Mudakir</t>
+  </si>
+  <si>
+    <t>Kusnanto</t>
+  </si>
+  <si>
+    <t>M. Lutfi</t>
+  </si>
+  <si>
+    <t>Nurohman</t>
+  </si>
+  <si>
+    <t>Muhammad Ali</t>
+  </si>
+  <si>
+    <t>Adi Kurniawan</t>
+  </si>
+  <si>
+    <t>M. Akrommudin</t>
+  </si>
+  <si>
+    <t>Muhammad Romadhon</t>
+  </si>
+  <si>
+    <t>Supriyanto</t>
+  </si>
+  <si>
+    <t>Nurul Khafidhin</t>
+  </si>
+  <si>
+    <t>Ulil Amri</t>
+  </si>
+  <si>
+    <t>Tenaga Administrasi</t>
+  </si>
+  <si>
+    <t>Petugas Penyapu Jalan</t>
+  </si>
+  <si>
+    <t>Petugas Kebersihan Depo/TPS</t>
+  </si>
+  <si>
+    <t>Tenaga Administrasi Bank Sampah</t>
+  </si>
+  <si>
+    <t>Petugas Kebersihan TPA</t>
+  </si>
+  <si>
+    <t>Petugas Angkutan Sampah</t>
+  </si>
+  <si>
+    <t>Petugas Pengelola Bank Sampah</t>
+  </si>
+  <si>
+    <t>Tenaga Analis Laboratorium</t>
+  </si>
+  <si>
+    <t>Petugas Taman</t>
+  </si>
+  <si>
+    <t>Tenaga Kebersihan Taman Hutan Raya (TAHURA)</t>
+  </si>
+  <si>
+    <t>Tenaga Kebersihan Perapihan Pohon</t>
+  </si>
+  <si>
+    <t>Petugas Pengelola IPAL</t>
+  </si>
+  <si>
+    <t>Petugas Truk Sedot Limbah</t>
+  </si>
+  <si>
+    <t>Petugas Jogokali</t>
+  </si>
+  <si>
+    <t>Sekretariat</t>
+  </si>
+  <si>
+    <t>KPS</t>
+  </si>
+  <si>
+    <t>PPKL-RTH</t>
   </si>
 </sst>
 </file>
@@ -49,7 +454,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -61,6 +466,15 @@
     </font>
     <font>
       <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b val="0"/>
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
@@ -104,12 +518,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="true">
       <protection locked="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+      <protection locked="true"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+      <protection locked="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
       <protection locked="true"/>
     </xf>
@@ -414,6 +836,17 @@
   </sheetPr>
   <dimension ref="A1:I900"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="true" style="0"/>
+    <col min="2" max="2" width="15" customWidth="true" style="0"/>
+    <col min="3" max="3" width="25" customWidth="true" style="0"/>
+    <col min="4" max="4" width="20" customWidth="true" style="0"/>
+    <col min="5" max="5" width="20" customWidth="true" style="0"/>
+    <col min="6" max="6" width="15" customWidth="true" style="0"/>
+    <col min="7" max="7" width="15" customWidth="true" style="0"/>
+    <col min="8" max="8" width="15" customWidth="true" style="0"/>
+    <col min="9" max="9" width="10" customWidth="true" style="0"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="2" t="s">
@@ -444,654 +877,1421 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-    </row>
-    <row r="27" spans="1:9">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
-    </row>
-    <row r="28" spans="1:9">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-    </row>
-    <row r="30" spans="1:9">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-    </row>
-    <row r="31" spans="1:9">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-    </row>
-    <row r="32" spans="1:9">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-    </row>
-    <row r="33" spans="1:9">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-    </row>
-    <row r="34" spans="1:9">
-      <c r="A34" s="1"/>
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
-    </row>
-    <row r="35" spans="1:9">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-    </row>
-    <row r="36" spans="1:9">
-      <c r="A36" s="1"/>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="1"/>
-      <c r="E36" s="1"/>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-    </row>
-    <row r="37" spans="1:9">
-      <c r="A37" s="1"/>
-      <c r="B37" s="1"/>
-      <c r="C37" s="1"/>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-    </row>
-    <row r="38" spans="1:9">
-      <c r="A38" s="1"/>
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-    </row>
-    <row r="39" spans="1:9">
-      <c r="A39" s="1"/>
-      <c r="B39" s="1"/>
-      <c r="C39" s="1"/>
-      <c r="D39" s="1"/>
-      <c r="E39" s="1"/>
-      <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
-      <c r="H39" s="1"/>
-      <c r="I39" s="1"/>
-    </row>
-    <row r="40" spans="1:9">
-      <c r="A40" s="1"/>
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-    </row>
-    <row r="41" spans="1:9">
-      <c r="A41" s="1"/>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
-      <c r="G41" s="1"/>
-      <c r="H41" s="1"/>
-      <c r="I41" s="1"/>
-    </row>
-    <row r="42" spans="1:9">
-      <c r="A42" s="1"/>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
-      <c r="G42" s="1"/>
-      <c r="H42" s="1"/>
-      <c r="I42" s="1"/>
-    </row>
-    <row r="43" spans="1:9">
-      <c r="A43" s="1"/>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
-      <c r="G43" s="1"/>
-      <c r="H43" s="1"/>
-      <c r="I43" s="1"/>
-    </row>
-    <row r="44" spans="1:9">
-      <c r="A44" s="1"/>
-      <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
-      <c r="G44" s="1"/>
-      <c r="H44" s="1"/>
-      <c r="I44" s="1"/>
-    </row>
-    <row r="45" spans="1:9">
-      <c r="A45" s="1"/>
-      <c r="B45" s="1"/>
-      <c r="C45" s="1"/>
-      <c r="D45" s="1"/>
-      <c r="E45" s="1"/>
-      <c r="F45" s="1"/>
-      <c r="G45" s="1"/>
-      <c r="H45" s="1"/>
-      <c r="I45" s="1"/>
-    </row>
-    <row r="46" spans="1:9">
-      <c r="A46" s="1"/>
-      <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
-      <c r="F46" s="1"/>
-      <c r="G46" s="1"/>
-      <c r="H46" s="1"/>
-      <c r="I46" s="1"/>
-    </row>
-    <row r="47" spans="1:9">
-      <c r="A47" s="1"/>
-      <c r="B47" s="1"/>
-      <c r="C47" s="1"/>
-      <c r="D47" s="1"/>
-      <c r="E47" s="1"/>
-      <c r="F47" s="1"/>
-      <c r="G47" s="1"/>
-      <c r="H47" s="1"/>
-      <c r="I47" s="1"/>
-    </row>
-    <row r="48" spans="1:9">
-      <c r="A48" s="1"/>
-      <c r="B48" s="1"/>
-      <c r="C48" s="1"/>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="1"/>
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-    </row>
-    <row r="49" spans="1:9">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
-      <c r="F49" s="1"/>
-      <c r="G49" s="1"/>
-      <c r="H49" s="1"/>
-      <c r="I49" s="1"/>
-    </row>
-    <row r="50" spans="1:9">
-      <c r="A50" s="1"/>
-      <c r="B50" s="1"/>
-      <c r="C50" s="1"/>
-      <c r="D50" s="1"/>
-      <c r="E50" s="1"/>
-      <c r="F50" s="1"/>
-      <c r="G50" s="1"/>
-      <c r="H50" s="1"/>
-      <c r="I50" s="1"/>
-    </row>
-    <row r="51" spans="1:9">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1"/>
-      <c r="E51" s="1"/>
-      <c r="F51" s="1"/>
-      <c r="G51" s="1"/>
-      <c r="H51" s="1"/>
-      <c r="I51" s="1"/>
-    </row>
-    <row r="52" spans="1:9">
-      <c r="A52" s="1"/>
-      <c r="B52" s="1"/>
-      <c r="C52" s="1"/>
-      <c r="D52" s="1"/>
-      <c r="E52" s="1"/>
-      <c r="F52" s="1"/>
-      <c r="G52" s="1"/>
-      <c r="H52" s="1"/>
-      <c r="I52" s="1"/>
-    </row>
-    <row r="53" spans="1:9">
-      <c r="A53" s="1"/>
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="1"/>
-      <c r="E53" s="1"/>
-      <c r="F53" s="1"/>
-      <c r="G53" s="1"/>
-      <c r="H53" s="1"/>
-      <c r="I53" s="1"/>
-    </row>
-    <row r="54" spans="1:9">
-      <c r="A54" s="1"/>
-      <c r="B54" s="1"/>
-      <c r="C54" s="1"/>
-      <c r="D54" s="1"/>
-      <c r="E54" s="1"/>
-      <c r="F54" s="1"/>
-      <c r="G54" s="1"/>
-      <c r="H54" s="1"/>
-      <c r="I54" s="1"/>
-    </row>
-    <row r="55" spans="1:9">
-      <c r="A55" s="1"/>
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="1"/>
-      <c r="E55" s="1"/>
-      <c r="F55" s="1"/>
-      <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
-      <c r="I55" s="1"/>
-    </row>
-    <row r="56" spans="1:9">
-      <c r="A56" s="1"/>
-      <c r="B56" s="1"/>
-      <c r="C56" s="1"/>
-      <c r="D56" s="1"/>
-      <c r="E56" s="1"/>
-      <c r="F56" s="1"/>
-      <c r="G56" s="1"/>
-      <c r="H56" s="1"/>
-      <c r="I56" s="1"/>
-    </row>
-    <row r="57" spans="1:9">
-      <c r="A57" s="1"/>
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="1"/>
-      <c r="E57" s="1"/>
-      <c r="F57" s="1"/>
-      <c r="G57" s="1"/>
-      <c r="H57" s="1"/>
-      <c r="I57" s="1"/>
-    </row>
-    <row r="58" spans="1:9">
-      <c r="A58" s="1"/>
-      <c r="B58" s="1"/>
-      <c r="C58" s="1"/>
-      <c r="D58" s="1"/>
-      <c r="E58" s="1"/>
-      <c r="F58" s="1"/>
-      <c r="G58" s="1"/>
-      <c r="H58" s="1"/>
-      <c r="I58" s="1"/>
-    </row>
-    <row r="59" spans="1:9">
-      <c r="A59" s="1"/>
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-      <c r="D59" s="1"/>
-      <c r="E59" s="1"/>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1"/>
-      <c r="H59" s="1"/>
-      <c r="I59" s="1"/>
-    </row>
-    <row r="60" spans="1:9">
-      <c r="A60" s="1"/>
-      <c r="B60" s="1"/>
-      <c r="C60" s="1"/>
-      <c r="D60" s="1"/>
-      <c r="E60" s="1"/>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1"/>
-      <c r="H60" s="1"/>
-      <c r="I60" s="1"/>
+    <row r="2" spans="1:9" customHeight="1" ht="20">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="4" t="e">
+        <f>YEAR(F2)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" customHeight="1" ht="20">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="4" t="e">
+        <f>YEAR(F3)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" customHeight="1" ht="20">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="4" t="e">
+        <f>YEAR(F4)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" customHeight="1" ht="20">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="4" t="e">
+        <f>YEAR(F5)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" customHeight="1" ht="20">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="4" t="e">
+        <f>YEAR(F6)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" customHeight="1" ht="20">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="4" t="e">
+        <f>YEAR(F7)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" customHeight="1" ht="20">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="4" t="e">
+        <f>YEAR(F8)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" customHeight="1" ht="20">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="4" t="e">
+        <f>YEAR(F9)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" customHeight="1" ht="20">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="4" t="e">
+        <f>YEAR(F10)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" customHeight="1" ht="20">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="4" t="e">
+        <f>YEAR(F11)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" customHeight="1" ht="20">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="4" t="e">
+        <f>YEAR(F12)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" customHeight="1" ht="20">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="4" t="e">
+        <f>YEAR(F13)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" customHeight="1" ht="20">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="4" t="e">
+        <f>YEAR(F14)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" customHeight="1" ht="20">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="4" t="e">
+        <f>YEAR(F15)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" customHeight="1" ht="20">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="4" t="e">
+        <f>YEAR(F16)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" customHeight="1" ht="20">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="4" t="e">
+        <f>YEAR(F17)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" customHeight="1" ht="20">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="4" t="e">
+        <f>YEAR(F18)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" customHeight="1" ht="20">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="4" t="e">
+        <f>YEAR(F19)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" customHeight="1" ht="20">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="4" t="e">
+        <f>YEAR(F20)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" customHeight="1" ht="20">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="4" t="e">
+        <f>YEAR(F21)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" customHeight="1" ht="20">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="4" t="e">
+        <f>YEAR(F22)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" customHeight="1" ht="20">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="4" t="e">
+        <f>YEAR(F23)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" customHeight="1" ht="20">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="4" t="e">
+        <f>YEAR(F24)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" customHeight="1" ht="20">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="4" t="e">
+        <f>YEAR(F25)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" customHeight="1" ht="20">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="4" t="e">
+        <f>YEAR(F26)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" customHeight="1" ht="20">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="4" t="e">
+        <f>YEAR(F27)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" customHeight="1" ht="20">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="4" t="e">
+        <f>YEAR(F28)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" customHeight="1" ht="20">
+      <c r="A29" s="3">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="4" t="e">
+        <f>YEAR(F29)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" customHeight="1" ht="20">
+      <c r="A30" s="3">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="4" t="e">
+        <f>YEAR(F30)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" customHeight="1" ht="20">
+      <c r="A31" s="3">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="4" t="e">
+        <f>YEAR(F31)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" customHeight="1" ht="20">
+      <c r="A32" s="3">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="4" t="e">
+        <f>YEAR(F32)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" customHeight="1" ht="20">
+      <c r="A33" s="3">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="4" t="e">
+        <f>YEAR(F33)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" customHeight="1" ht="20">
+      <c r="A34" s="3">
+        <v>33</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="4" t="e">
+        <f>YEAR(F34)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" customHeight="1" ht="20">
+      <c r="A35" s="3">
+        <v>34</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="4" t="e">
+        <f>YEAR(F35)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" customHeight="1" ht="20">
+      <c r="A36" s="3">
+        <v>35</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="4" t="e">
+        <f>YEAR(F36)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" customHeight="1" ht="20">
+      <c r="A37" s="3">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="4" t="e">
+        <f>YEAR(F37)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" customHeight="1" ht="20">
+      <c r="A38" s="3">
+        <v>37</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="4" t="e">
+        <f>YEAR(F38)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" customHeight="1" ht="20">
+      <c r="A39" s="3">
+        <v>38</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="4" t="e">
+        <f>YEAR(F39)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" customHeight="1" ht="20">
+      <c r="A40" s="3">
+        <v>39</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="4" t="e">
+        <f>YEAR(F40)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" customHeight="1" ht="20">
+      <c r="A41" s="3">
+        <v>40</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="4" t="e">
+        <f>YEAR(F41)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" customHeight="1" ht="20">
+      <c r="A42" s="3">
+        <v>41</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="4" t="e">
+        <f>YEAR(F42)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" customHeight="1" ht="20">
+      <c r="A43" s="3">
+        <v>42</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="4" t="e">
+        <f>YEAR(F43)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" customHeight="1" ht="20">
+      <c r="A44" s="3">
+        <v>43</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="4" t="e">
+        <f>YEAR(F44)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" customHeight="1" ht="20">
+      <c r="A45" s="3">
+        <v>44</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="4" t="e">
+        <f>YEAR(F45)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" customHeight="1" ht="20">
+      <c r="A46" s="3">
+        <v>45</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="4" t="e">
+        <f>YEAR(F46)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" customHeight="1" ht="20">
+      <c r="A47" s="3">
+        <v>46</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="4" t="e">
+        <f>YEAR(F47)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" customHeight="1" ht="20">
+      <c r="A48" s="3">
+        <v>47</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="4" t="e">
+        <f>YEAR(F48)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" customHeight="1" ht="20">
+      <c r="A49" s="3">
+        <v>48</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="4" t="e">
+        <f>YEAR(F49)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" customHeight="1" ht="20">
+      <c r="A50" s="3">
+        <v>49</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="4" t="e">
+        <f>YEAR(F50)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" customHeight="1" ht="20">
+      <c r="A51" s="3">
+        <v>50</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="4" t="e">
+        <f>YEAR(F51)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" customHeight="1" ht="20">
+      <c r="A52" s="3">
+        <v>51</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="4" t="e">
+        <f>YEAR(F52)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" customHeight="1" ht="20">
+      <c r="A53" s="3">
+        <v>52</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="4" t="e">
+        <f>YEAR(F53)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" customHeight="1" ht="20">
+      <c r="A54" s="3">
+        <v>53</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="4" t="e">
+        <f>YEAR(F54)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" customHeight="1" ht="20">
+      <c r="A55" s="3">
+        <v>54</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="4" t="e">
+        <f>YEAR(F55)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" customHeight="1" ht="20">
+      <c r="A56" s="3">
+        <v>55</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="4" t="e">
+        <f>YEAR(F56)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" customHeight="1" ht="20">
+      <c r="A57" s="3">
+        <v>56</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="4" t="e">
+        <f>YEAR(F57)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" customHeight="1" ht="20">
+      <c r="A58" s="3">
+        <v>57</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+      <c r="I58" s="4" t="e">
+        <f>YEAR(F58)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" customHeight="1" ht="20">
+      <c r="A59" s="3">
+        <v>58</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+      <c r="I59" s="4" t="e">
+        <f>YEAR(F59)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" customHeight="1" ht="20">
+      <c r="A60" s="3">
+        <v>59</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="4" t="e">
+        <f>YEAR(F60)</f>
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="61" spans="1:9">
       <c r="A61" s="1"/>
@@ -10335,6 +11535,657 @@
     </row>
   </sheetData>
   <sheetProtection password="9D39" sheet="1"/>
+  <dataValidations count="295">
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D2">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E2">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F2"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G2"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H2">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D3">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E3">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F3"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G3"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H3">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D4">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E4">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F4"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G4"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H4">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D5">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E5">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F5"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G5"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H5">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D6">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E6">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F6"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G6"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H6">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D7">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E7">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F7"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G7"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H7">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D8">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E8">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F8"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G8"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H8">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D9">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E9">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F9"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G9"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H9">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D10">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E10">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F10"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G10"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H10">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D11">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E11">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F11"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G11"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H11">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D12">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E12">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F12"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G12"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H12">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D13">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E13">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F13"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G13"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H13">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D14">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E14">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F14"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G14"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H14">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D15">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E15">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F15"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G15"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H15">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D16">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E16">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F16"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G16"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H16">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D17">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E17">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F17"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G17"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H17">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D18">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E18">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F18"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G18"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H18">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D19">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E19">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F19"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G19"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H19">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D20">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E20">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F20"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G20"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H20">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D21">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E21">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F21"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G21"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H21">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D22">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E22">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F22"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G22"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H22">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D23">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E23">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F23"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G23"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H23">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D24">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E24">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F24"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G24"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H24">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D25">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E25">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F25"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G25"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H25">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D26">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E26">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F26"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G26"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H26">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D27">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E27">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F27"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G27"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H27">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D28">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E28">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F28"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G28"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H28">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D29">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E29">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F29"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G29"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H29">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D30">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E30">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F30"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G30"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H30">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D31">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E31">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F31"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G31"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H31">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D32">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E32">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F32"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G32"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H32">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D33">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E33">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F33"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G33"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H33">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D34">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E34">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F34"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G34"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H34">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D35">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E35">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F35"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G35"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H35">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D36">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E36">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F36"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G36"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H36">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D37">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E37">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F37"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G37"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H37">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D38">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E38">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F38"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G38"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H38">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D39">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E39">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F39"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G39"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H39">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D40">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E40">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F40"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G40"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H40">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D41">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E41">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F41"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G41"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H41">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D42">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E42">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F42"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G42"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H42">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D43">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E43">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F43"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G43"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H43">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D44">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E44">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F44"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G44"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H44">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D45">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E45">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F45"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G45"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H45">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D46">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E46">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F46"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G46"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H46">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D47">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E47">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F47"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G47"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H47">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D48">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E48">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F48"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G48"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H48">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D49">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E49">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F49"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G49"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H49">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D50">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E50">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F50"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G50"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H50">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D51">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E51">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F51"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G51"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H51">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D52">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E52">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F52"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G52"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H52">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D53">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E53">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F53"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G53"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H53">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D54">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E54">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F54"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G54"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H54">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D55">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E55">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F55"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G55"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H55">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D56">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E56">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F56"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G56"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H56">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D57">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E57">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F57"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G57"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H57">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D58">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E58">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F58"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G58"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H58">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D59">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E59">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F59"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G59"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H59">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D60">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E60">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F60"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G60"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H60">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>

</xml_diff>

<commit_message>
fix: fitur nomor sk
</commit_message>
<xml_diff>
--- a/public/template/template_riwayat_kerja.xlsx
+++ b/public/template/template_riwayat_kerja.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="146">
   <si>
     <t>No</t>
   </si>
@@ -221,6 +221,9 @@
     <t>PG260129995530</t>
   </si>
   <si>
+    <t>PG260709582949</t>
+  </si>
+  <si>
     <t>Fajar Aji Kusuma</t>
   </si>
   <si>
@@ -396,6 +399,9 @@
   </si>
   <si>
     <t>Ulil Amri</t>
+  </si>
+  <si>
+    <t>Isna Septiana</t>
   </si>
   <si>
     <t>Tenaga Administrasi</t>
@@ -885,13 +891,13 @@
         <v>9</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
@@ -909,13 +915,13 @@
         <v>10</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -933,13 +939,13 @@
         <v>11</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -957,13 +963,13 @@
         <v>12</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -981,13 +987,13 @@
         <v>13</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -1005,13 +1011,13 @@
         <v>14</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -1029,13 +1035,13 @@
         <v>15</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
@@ -1053,13 +1059,13 @@
         <v>16</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -1077,13 +1083,13 @@
         <v>17</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -1101,13 +1107,13 @@
         <v>18</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
@@ -1125,13 +1131,13 @@
         <v>19</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -1149,13 +1155,13 @@
         <v>20</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
@@ -1173,13 +1179,13 @@
         <v>21</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -1197,13 +1203,13 @@
         <v>22</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
@@ -1221,13 +1227,13 @@
         <v>23</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -1245,13 +1251,13 @@
         <v>24</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
@@ -1269,13 +1275,13 @@
         <v>25</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -1293,13 +1299,13 @@
         <v>26</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -1317,13 +1323,13 @@
         <v>27</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -1341,13 +1347,13 @@
         <v>28</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -1365,13 +1371,13 @@
         <v>29</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -1389,13 +1395,13 @@
         <v>30</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
@@ -1413,13 +1419,13 @@
         <v>31</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -1437,13 +1443,13 @@
         <v>32</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -1461,13 +1467,13 @@
         <v>33</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -1485,13 +1491,13 @@
         <v>34</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -1509,13 +1515,13 @@
         <v>35</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -1533,13 +1539,13 @@
         <v>36</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -1557,13 +1563,13 @@
         <v>37</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
@@ -1581,13 +1587,13 @@
         <v>38</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -1605,13 +1611,13 @@
         <v>39</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
@@ -1629,13 +1635,13 @@
         <v>40</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
@@ -1653,13 +1659,13 @@
         <v>41</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -1677,13 +1683,13 @@
         <v>42</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -1701,13 +1707,13 @@
         <v>43</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -1725,13 +1731,13 @@
         <v>44</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -1749,13 +1755,13 @@
         <v>45</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
@@ -1773,13 +1779,13 @@
         <v>46</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -1797,13 +1803,13 @@
         <v>47</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -1821,13 +1827,13 @@
         <v>48</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -1845,13 +1851,13 @@
         <v>49</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -1869,13 +1875,13 @@
         <v>50</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
@@ -1893,13 +1899,13 @@
         <v>51</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -1917,13 +1923,13 @@
         <v>52</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -1941,13 +1947,13 @@
         <v>53</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
@@ -1965,13 +1971,13 @@
         <v>54</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -1989,13 +1995,13 @@
         <v>55</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -2013,13 +2019,13 @@
         <v>56</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -2037,13 +2043,13 @@
         <v>57</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -2061,13 +2067,13 @@
         <v>58</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -2085,13 +2091,13 @@
         <v>59</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
@@ -2109,13 +2115,13 @@
         <v>60</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -2133,13 +2139,13 @@
         <v>61</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
@@ -2157,13 +2163,13 @@
         <v>62</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -2181,13 +2187,13 @@
         <v>63</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -2205,13 +2211,13 @@
         <v>64</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -2229,13 +2235,13 @@
         <v>65</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3"/>
@@ -2253,13 +2259,13 @@
         <v>66</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
@@ -2277,13 +2283,13 @@
         <v>67</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
@@ -2293,16 +2299,29 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="61" spans="1:9">
-      <c r="A61" s="1"/>
-      <c r="B61" s="1"/>
-      <c r="C61" s="1"/>
-      <c r="D61" s="1"/>
-      <c r="E61" s="1"/>
-      <c r="F61" s="1"/>
-      <c r="G61" s="1"/>
-      <c r="H61" s="1"/>
-      <c r="I61" s="1"/>
+    <row r="61" spans="1:9" customHeight="1" ht="20">
+      <c r="A61" s="3">
+        <v>60</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
+      <c r="I61" s="4" t="e">
+        <f>YEAR(F61)</f>
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="62" spans="1:9">
       <c r="A62" s="1"/>
@@ -11535,7 +11554,7 @@
     </row>
   </sheetData>
   <sheetProtection password="9D39" sheet="1"/>
-  <dataValidations count="295">
+  <dataValidations count="300">
     <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D2">
       <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
     </dataValidation>
@@ -12183,6 +12202,17 @@
     <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F60"/>
     <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G60"/>
     <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H60">
+      <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="D61">
+      <formula1>"Tenaga Administrasi,Tenaga Kebersihan Taman Hutan Raya (TAHURA),Tenaga Kebersihan Perapihan Pohon,Petugas Keamanan,Pengemudi Angkutan Sampah,Kru Angkutan Sampah,Petugas Depo,Petugas Patroli,Tenaga Administrasi Bank Sampah,Petugas Pengelola Bank Sampah,Petugas Jaga Malam Bank Sampah,Petugas TPA,Petugas Jaga Malam TPA,Petugas Penyapu Jalan,Petugas Kebersihan Depo/TPS,Petugas Angkutan Sampah,Petugas Kebersihan TPA,Tenaga Pengelola Bank Sampah Induk,Petugas Jogokali,Tenaga Analis Laboratorium,Petugas Taman,Petugas Pengelola IPAL,Petugas Truk Sedot Limbah"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="E61">
+      <formula1>"Sekretariat,Taling,KPS,PPKL-RTH"</formula1>
+    </dataValidation>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F61"/>
+    <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="G61"/>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="H61">
       <formula1>"Kontak Dinas,Kontak Walikota"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>